<commit_message>
UAT set 2: use aymish143 inbox
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRRBvkKjt3A9PgQv7tKcVq
</commit_message>
<xml_diff>
--- a/project/sample-imports/doctors-uat2.xlsx
+++ b/project/sample-imports/doctors-uat2.xlsx
@@ -46,7 +46,7 @@
     <t>Dlamini</t>
   </si>
   <si>
-    <t>maziyamayo7+uat2doctor1@gmail.com</t>
+    <t>aymish143+uat2doctor1@gmail.com</t>
   </si>
   <si>
     <t>0716660001</t>
@@ -70,7 +70,7 @@
     <t>Mabaso</t>
   </si>
   <si>
-    <t>makabmahlalela+uat2doctor2@gmail.com</t>
+    <t>aymish143+uat2doctor2@gmail.com</t>
   </si>
   <si>
     <t>0716660002</t>
@@ -91,7 +91,7 @@
     <t>Pretorius</t>
   </si>
   <si>
-    <t>maziyamayo7+uat2doctor3@gmail.com</t>
+    <t>aymish143+uat2doctor3@gmail.com</t>
   </si>
   <si>
     <t>0716660003</t>
@@ -112,7 +112,7 @@
     <t>Modise</t>
   </si>
   <si>
-    <t>makabmahlalela+uat2doctor4@gmail.com</t>
+    <t>aymish143+uat2doctor4@gmail.com</t>
   </si>
   <si>
     <t>0716660004</t>
@@ -133,7 +133,7 @@
     <t>Shabalala</t>
   </si>
   <si>
-    <t>maziyamayo7+uat2doctor5@gmail.com</t>
+    <t>aymish143+uat2doctor5@gmail.com</t>
   </si>
   <si>
     <t>0716660005</t>
@@ -683,6 +683,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>